<commit_message>
Add techincal roadmap ppt and Energy meter doc
</commit_message>
<xml_diff>
--- a/Docs/Gantt Chart.xlsx
+++ b/Docs/Gantt Chart.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\DOCUMENTATIONS\EV-battery-packs\Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\DOCUMENTATIONS\battery-pack-engineering\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{332A6172-B2A6-47FA-907A-4B9BB9EA2084}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A7350C5-AAB5-48C7-8B22-07FC7CC2FDE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="80">
   <si>
     <t>Insert new rows ABOVE this one</t>
   </si>
@@ -285,6 +285,12 @@
   </si>
   <si>
     <t>4S Series Welding, BMS Wiring &amp; Heat Shrink</t>
+  </si>
+  <si>
+    <t>Outdoor Solar Charge &amp; Cycle Validation</t>
+  </si>
+  <si>
+    <t>Completed 3 days continous outdoor test: connected directly to solar panel.</t>
   </si>
 </sst>
 </file>
@@ -1200,53 +1206,53 @@
     <xf numFmtId="165" fontId="32" fillId="10" borderId="0" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="19" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="19" fillId="2" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="19" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="27" fillId="0" borderId="0" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="8" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="11" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="19" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="19" fillId="2" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="19" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="166" fontId="27" fillId="0" borderId="0" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="8" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="13">
@@ -1585,7 +1591,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp1.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Scroll" dx="26" fmlaLink="$R$2" horiz="1" max="10" min="1" page="0" val="8"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Scroll" dx="26" fmlaLink="$R$2" horiz="1" max="20" min="1" page="0" val="8"/>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1966,7 +1972,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BW44"/>
+  <dimension ref="A1:BW45"/>
   <sheetFormatPr defaultColWidth="8.69921875" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.69921875" style="13" customWidth="1"/>
@@ -1992,61 +1998,61 @@
       <c r="F1" s="21"/>
       <c r="G1" s="21"/>
       <c r="I1" s="1"/>
-      <c r="J1" s="119" t="s">
+      <c r="J1" s="117" t="s">
         <v>20</v>
       </c>
-      <c r="K1" s="120"/>
-      <c r="L1" s="120"/>
-      <c r="M1" s="120"/>
-      <c r="N1" s="120"/>
-      <c r="O1" s="120"/>
-      <c r="P1" s="120"/>
+      <c r="K1" s="118"/>
+      <c r="L1" s="118"/>
+      <c r="M1" s="118"/>
+      <c r="N1" s="118"/>
+      <c r="O1" s="118"/>
+      <c r="P1" s="118"/>
       <c r="Q1" s="24"/>
-      <c r="R1" s="118">
+      <c r="R1" s="115">
         <f>DATE(2026,6,12)</f>
         <v>46185</v>
       </c>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="117"/>
-      <c r="V1" s="117"/>
-      <c r="W1" s="117"/>
-      <c r="X1" s="117"/>
-      <c r="Y1" s="117"/>
-      <c r="Z1" s="117"/>
-      <c r="AA1" s="117"/>
+      <c r="S1" s="116"/>
+      <c r="T1" s="116"/>
+      <c r="U1" s="116"/>
+      <c r="V1" s="116"/>
+      <c r="W1" s="116"/>
+      <c r="X1" s="116"/>
+      <c r="Y1" s="116"/>
+      <c r="Z1" s="116"/>
+      <c r="AA1" s="116"/>
     </row>
     <row r="2" spans="1:75" ht="30" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="B2" s="112" t="s">
+      <c r="B2" s="126" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="112"/>
+      <c r="C2" s="126"/>
       <c r="D2" s="22"/>
       <c r="E2" s="23"/>
       <c r="F2" s="22"/>
       <c r="G2" s="22"/>
-      <c r="J2" s="119" t="s">
+      <c r="J2" s="117" t="s">
         <v>21</v>
       </c>
-      <c r="K2" s="120"/>
-      <c r="L2" s="120"/>
-      <c r="M2" s="120"/>
-      <c r="N2" s="120"/>
-      <c r="O2" s="120"/>
-      <c r="P2" s="120"/>
+      <c r="K2" s="118"/>
+      <c r="L2" s="118"/>
+      <c r="M2" s="118"/>
+      <c r="N2" s="118"/>
+      <c r="O2" s="118"/>
+      <c r="P2" s="118"/>
       <c r="Q2" s="24"/>
-      <c r="R2" s="116">
+      <c r="R2" s="127">
         <v>8</v>
       </c>
-      <c r="S2" s="117"/>
-      <c r="T2" s="117"/>
-      <c r="U2" s="117"/>
-      <c r="V2" s="117"/>
-      <c r="W2" s="117"/>
-      <c r="X2" s="117"/>
-      <c r="Y2" s="117"/>
-      <c r="Z2" s="117"/>
-      <c r="AA2" s="117"/>
+      <c r="S2" s="116"/>
+      <c r="T2" s="116"/>
+      <c r="U2" s="116"/>
+      <c r="V2" s="116"/>
+      <c r="W2" s="116"/>
+      <c r="X2" s="116"/>
+      <c r="Y2" s="116"/>
+      <c r="Z2" s="116"/>
+      <c r="AA2" s="116"/>
     </row>
     <row r="3" spans="1:75" s="26" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="13"/>
@@ -2058,86 +2064,86 @@
       <c r="A4" s="14"/>
       <c r="B4" s="29"/>
       <c r="E4" s="30"/>
-      <c r="J4" s="115">
+      <c r="J4" s="114">
         <f>J5</f>
         <v>46230</v>
       </c>
-      <c r="K4" s="113"/>
-      <c r="L4" s="113"/>
-      <c r="M4" s="113"/>
-      <c r="N4" s="113"/>
-      <c r="O4" s="113"/>
-      <c r="P4" s="113"/>
-      <c r="Q4" s="113">
+      <c r="K4" s="112"/>
+      <c r="L4" s="112"/>
+      <c r="M4" s="112"/>
+      <c r="N4" s="112"/>
+      <c r="O4" s="112"/>
+      <c r="P4" s="112"/>
+      <c r="Q4" s="112">
         <f>Q5</f>
         <v>46237</v>
       </c>
-      <c r="R4" s="113"/>
-      <c r="S4" s="113"/>
-      <c r="T4" s="113"/>
-      <c r="U4" s="113"/>
-      <c r="V4" s="113"/>
-      <c r="W4" s="113"/>
-      <c r="X4" s="113">
+      <c r="R4" s="112"/>
+      <c r="S4" s="112"/>
+      <c r="T4" s="112"/>
+      <c r="U4" s="112"/>
+      <c r="V4" s="112"/>
+      <c r="W4" s="112"/>
+      <c r="X4" s="112">
         <f>X5</f>
         <v>46244</v>
       </c>
-      <c r="Y4" s="113"/>
-      <c r="Z4" s="113"/>
-      <c r="AA4" s="113"/>
-      <c r="AB4" s="113"/>
-      <c r="AC4" s="113"/>
-      <c r="AD4" s="113"/>
-      <c r="AE4" s="113">
+      <c r="Y4" s="112"/>
+      <c r="Z4" s="112"/>
+      <c r="AA4" s="112"/>
+      <c r="AB4" s="112"/>
+      <c r="AC4" s="112"/>
+      <c r="AD4" s="112"/>
+      <c r="AE4" s="112">
         <f>AE5</f>
         <v>46251</v>
       </c>
-      <c r="AF4" s="113"/>
-      <c r="AG4" s="113"/>
-      <c r="AH4" s="113"/>
-      <c r="AI4" s="113"/>
-      <c r="AJ4" s="113"/>
-      <c r="AK4" s="113"/>
-      <c r="AL4" s="113">
+      <c r="AF4" s="112"/>
+      <c r="AG4" s="112"/>
+      <c r="AH4" s="112"/>
+      <c r="AI4" s="112"/>
+      <c r="AJ4" s="112"/>
+      <c r="AK4" s="112"/>
+      <c r="AL4" s="112">
         <f>AL5</f>
         <v>46258</v>
       </c>
-      <c r="AM4" s="113"/>
-      <c r="AN4" s="113"/>
-      <c r="AO4" s="113"/>
-      <c r="AP4" s="113"/>
-      <c r="AQ4" s="113"/>
-      <c r="AR4" s="113"/>
-      <c r="AS4" s="113">
+      <c r="AM4" s="112"/>
+      <c r="AN4" s="112"/>
+      <c r="AO4" s="112"/>
+      <c r="AP4" s="112"/>
+      <c r="AQ4" s="112"/>
+      <c r="AR4" s="112"/>
+      <c r="AS4" s="112">
         <f>AS5</f>
         <v>46265</v>
       </c>
-      <c r="AT4" s="113"/>
-      <c r="AU4" s="113"/>
-      <c r="AV4" s="113"/>
-      <c r="AW4" s="113"/>
-      <c r="AX4" s="113"/>
-      <c r="AY4" s="113"/>
-      <c r="AZ4" s="113">
+      <c r="AT4" s="112"/>
+      <c r="AU4" s="112"/>
+      <c r="AV4" s="112"/>
+      <c r="AW4" s="112"/>
+      <c r="AX4" s="112"/>
+      <c r="AY4" s="112"/>
+      <c r="AZ4" s="112">
         <f>AZ5</f>
         <v>46272</v>
       </c>
-      <c r="BA4" s="113"/>
-      <c r="BB4" s="113"/>
-      <c r="BC4" s="113"/>
-      <c r="BD4" s="113"/>
-      <c r="BE4" s="113"/>
-      <c r="BF4" s="113"/>
-      <c r="BG4" s="113">
+      <c r="BA4" s="112"/>
+      <c r="BB4" s="112"/>
+      <c r="BC4" s="112"/>
+      <c r="BD4" s="112"/>
+      <c r="BE4" s="112"/>
+      <c r="BF4" s="112"/>
+      <c r="BG4" s="112">
         <f>BG5</f>
         <v>46279</v>
       </c>
-      <c r="BH4" s="113"/>
-      <c r="BI4" s="113"/>
-      <c r="BJ4" s="113"/>
-      <c r="BK4" s="113"/>
-      <c r="BL4" s="113"/>
-      <c r="BM4" s="114"/>
+      <c r="BH4" s="112"/>
+      <c r="BI4" s="112"/>
+      <c r="BJ4" s="112"/>
+      <c r="BK4" s="112"/>
+      <c r="BL4" s="112"/>
+      <c r="BM4" s="113"/>
     </row>
     <row r="5" spans="1:75" s="26" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="121"/>
@@ -2147,16 +2153,16 @@
       <c r="C5" s="124" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="110" t="s">
+      <c r="D5" s="119" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="110" t="s">
+      <c r="E5" s="119" t="s">
         <v>3</v>
       </c>
-      <c r="F5" s="110" t="s">
+      <c r="F5" s="119" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="110" t="s">
+      <c r="G5" s="119" t="s">
         <v>24</v>
       </c>
       <c r="J5" s="31">
@@ -2388,10 +2394,10 @@
       <c r="A6" s="121"/>
       <c r="B6" s="123"/>
       <c r="C6" s="125"/>
-      <c r="D6" s="111"/>
-      <c r="E6" s="111"/>
-      <c r="F6" s="111"/>
-      <c r="G6" s="111"/>
+      <c r="D6" s="120"/>
+      <c r="E6" s="120"/>
+      <c r="F6" s="120"/>
+      <c r="G6" s="120"/>
       <c r="J6" s="34" t="str">
         <f t="shared" ref="J6:AO6" si="3">LEFT(TEXT(J5,"ddd"),1)</f>
         <v>M</v>
@@ -2700,7 +2706,7 @@
       <c r="G8" s="44"/>
       <c r="H8" s="17"/>
       <c r="I8" s="5" t="str">
-        <f t="shared" ref="I8:I41" si="5">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <f t="shared" ref="I8:I42" si="5">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
       <c r="J8" s="45"/>
@@ -4640,13 +4646,13 @@
     </row>
     <row r="32" spans="1:75" s="46" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="13"/>
-      <c r="B32" s="126" t="s">
+      <c r="B32" s="110" t="s">
         <v>76</v>
       </c>
       <c r="C32" s="67" t="s">
         <v>28</v>
       </c>
-      <c r="D32" s="127">
+      <c r="D32" s="111">
         <v>1</v>
       </c>
       <c r="E32" s="69">
@@ -4721,13 +4727,13 @@
     </row>
     <row r="33" spans="1:65" s="46" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="13"/>
-      <c r="B33" s="126" t="s">
+      <c r="B33" s="110" t="s">
         <v>77</v>
       </c>
       <c r="C33" s="67" t="s">
         <v>28</v>
       </c>
-      <c r="D33" s="127">
+      <c r="D33" s="111">
         <v>1</v>
       </c>
       <c r="E33" s="69">
@@ -4802,19 +4808,28 @@
     </row>
     <row r="34" spans="1:65" s="46" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="13"/>
-      <c r="B34" s="70" t="s">
-        <v>23</v>
-      </c>
-      <c r="C34" s="71"/>
-      <c r="D34" s="72"/>
-      <c r="E34" s="73"/>
-      <c r="F34" s="74"/>
-      <c r="G34" s="74"/>
+      <c r="B34" s="110" t="s">
+        <v>78</v>
+      </c>
+      <c r="C34" s="67" t="s">
+        <v>28</v>
+      </c>
+      <c r="D34" s="111">
+        <v>1</v>
+      </c>
+      <c r="E34" s="69">
+        <f>DATE(2026,9,11)</f>
+        <v>46276</v>
+      </c>
+      <c r="F34" s="69">
+        <f>DATE(2026,9,14)</f>
+        <v>46279</v>
+      </c>
+      <c r="G34" s="107" t="s">
+        <v>79</v>
+      </c>
       <c r="H34" s="17"/>
-      <c r="I34" s="5" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
+      <c r="I34" s="5"/>
       <c r="J34" s="75"/>
       <c r="K34" s="75"/>
       <c r="L34" s="75"/>
@@ -4874,77 +4889,75 @@
     </row>
     <row r="35" spans="1:65" s="46" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="13"/>
-      <c r="B35" s="108"/>
-      <c r="C35" s="76" t="s">
-        <v>28</v>
-      </c>
-      <c r="D35" s="77">
-        <v>0.25</v>
-      </c>
-      <c r="E35" s="78"/>
-      <c r="F35" s="78"/>
-      <c r="G35" s="109"/>
+      <c r="B35" s="70" t="s">
+        <v>23</v>
+      </c>
+      <c r="C35" s="71"/>
+      <c r="D35" s="72"/>
+      <c r="E35" s="73"/>
+      <c r="F35" s="74"/>
+      <c r="G35" s="74"/>
       <c r="H35" s="17"/>
       <c r="I35" s="5" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J35" s="50"/>
-      <c r="K35" s="50"/>
-      <c r="L35" s="50"/>
-      <c r="M35" s="50"/>
-      <c r="N35" s="50"/>
-      <c r="O35" s="50"/>
-      <c r="P35" s="50"/>
-      <c r="Q35" s="50"/>
-      <c r="R35" s="50"/>
-      <c r="S35" s="50"/>
-      <c r="T35" s="50"/>
-      <c r="U35" s="50"/>
-      <c r="V35" s="50"/>
-      <c r="W35" s="50"/>
-      <c r="X35" s="50"/>
-      <c r="Y35" s="50"/>
-      <c r="Z35" s="50"/>
-      <c r="AA35" s="50"/>
-      <c r="AB35" s="50"/>
-      <c r="AC35" s="50"/>
-      <c r="AD35" s="50"/>
-      <c r="AE35" s="50"/>
-      <c r="AF35" s="50"/>
-      <c r="AG35" s="50"/>
-      <c r="AH35" s="50"/>
-      <c r="AI35" s="50"/>
-      <c r="AJ35" s="50"/>
-      <c r="AK35" s="50"/>
-      <c r="AL35" s="50"/>
-      <c r="AM35" s="50"/>
-      <c r="AN35" s="50"/>
-      <c r="AO35" s="50"/>
-      <c r="AP35" s="50"/>
-      <c r="AQ35" s="50"/>
-      <c r="AR35" s="50"/>
-      <c r="AS35" s="50"/>
-      <c r="AT35" s="50"/>
-      <c r="AU35" s="50"/>
-      <c r="AV35" s="50"/>
-      <c r="AW35" s="50"/>
-      <c r="AX35" s="50"/>
-      <c r="AY35" s="50"/>
-      <c r="AZ35" s="50"/>
-      <c r="BA35" s="50"/>
-      <c r="BB35" s="50"/>
-      <c r="BC35" s="50"/>
-      <c r="BD35" s="50"/>
-      <c r="BE35" s="50"/>
-      <c r="BF35" s="50"/>
-      <c r="BG35" s="50"/>
-      <c r="BH35" s="50"/>
-      <c r="BI35" s="50"/>
-      <c r="BJ35" s="50"/>
-      <c r="BK35" s="50"/>
-      <c r="BL35" s="50"/>
-      <c r="BM35" s="50"/>
+      <c r="J35" s="75"/>
+      <c r="K35" s="75"/>
+      <c r="L35" s="75"/>
+      <c r="M35" s="75"/>
+      <c r="N35" s="75"/>
+      <c r="O35" s="75"/>
+      <c r="P35" s="75"/>
+      <c r="Q35" s="75"/>
+      <c r="R35" s="75"/>
+      <c r="S35" s="75"/>
+      <c r="T35" s="75"/>
+      <c r="U35" s="75"/>
+      <c r="V35" s="75"/>
+      <c r="W35" s="75"/>
+      <c r="X35" s="75"/>
+      <c r="Y35" s="75"/>
+      <c r="Z35" s="75"/>
+      <c r="AA35" s="75"/>
+      <c r="AB35" s="75"/>
+      <c r="AC35" s="75"/>
+      <c r="AD35" s="75"/>
+      <c r="AE35" s="75"/>
+      <c r="AF35" s="75"/>
+      <c r="AG35" s="75"/>
+      <c r="AH35" s="75"/>
+      <c r="AI35" s="75"/>
+      <c r="AJ35" s="75"/>
+      <c r="AK35" s="75"/>
+      <c r="AL35" s="75"/>
+      <c r="AM35" s="75"/>
+      <c r="AN35" s="75"/>
+      <c r="AO35" s="75"/>
+      <c r="AP35" s="75"/>
+      <c r="AQ35" s="75"/>
+      <c r="AR35" s="75"/>
+      <c r="AS35" s="75"/>
+      <c r="AT35" s="75"/>
+      <c r="AU35" s="75"/>
+      <c r="AV35" s="75"/>
+      <c r="AW35" s="75"/>
+      <c r="AX35" s="75"/>
+      <c r="AY35" s="75"/>
+      <c r="AZ35" s="75"/>
+      <c r="BA35" s="75"/>
+      <c r="BB35" s="75"/>
+      <c r="BC35" s="75"/>
+      <c r="BD35" s="75"/>
+      <c r="BE35" s="75"/>
+      <c r="BF35" s="75"/>
+      <c r="BG35" s="75"/>
+      <c r="BH35" s="75"/>
+      <c r="BI35" s="75"/>
+      <c r="BJ35" s="75"/>
+      <c r="BK35" s="75"/>
+      <c r="BL35" s="75"/>
+      <c r="BM35" s="75"/>
     </row>
     <row r="36" spans="1:65" s="46" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="13"/>
@@ -5027,7 +5040,7 @@
         <v>28</v>
       </c>
       <c r="D37" s="77">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="E37" s="78"/>
       <c r="F37" s="78"/>
@@ -5101,7 +5114,7 @@
         <v>28</v>
       </c>
       <c r="D38" s="77">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="E38" s="78"/>
       <c r="F38" s="78"/>
@@ -5175,7 +5188,7 @@
         <v>28</v>
       </c>
       <c r="D39" s="77">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="E39" s="78"/>
       <c r="F39" s="78"/>
@@ -5244,156 +5257,230 @@
     </row>
     <row r="40" spans="1:65" s="46" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="13"/>
-      <c r="B40" s="79"/>
-      <c r="C40" s="80"/>
-      <c r="D40" s="81"/>
-      <c r="E40" s="82"/>
-      <c r="F40" s="82"/>
-      <c r="G40" s="82"/>
+      <c r="B40" s="108"/>
+      <c r="C40" s="76" t="s">
+        <v>28</v>
+      </c>
+      <c r="D40" s="77">
+        <v>0.5</v>
+      </c>
+      <c r="E40" s="78"/>
+      <c r="F40" s="78"/>
+      <c r="G40" s="109"/>
       <c r="H40" s="17"/>
       <c r="I40" s="5" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J40" s="45"/>
-      <c r="K40" s="45"/>
-      <c r="L40" s="45"/>
-      <c r="M40" s="45"/>
-      <c r="N40" s="45"/>
-      <c r="O40" s="45"/>
-      <c r="P40" s="45"/>
-      <c r="Q40" s="45"/>
-      <c r="R40" s="45"/>
-      <c r="S40" s="45"/>
-      <c r="T40" s="45"/>
-      <c r="U40" s="45"/>
-      <c r="V40" s="45"/>
-      <c r="W40" s="45"/>
-      <c r="X40" s="45"/>
-      <c r="Y40" s="45"/>
-      <c r="Z40" s="45"/>
-      <c r="AA40" s="45"/>
-      <c r="AB40" s="45"/>
-      <c r="AC40" s="45"/>
-      <c r="AD40" s="45"/>
-      <c r="AE40" s="45"/>
-      <c r="AF40" s="45"/>
-      <c r="AG40" s="45"/>
-      <c r="AH40" s="45"/>
-      <c r="AI40" s="45"/>
-      <c r="AJ40" s="45"/>
-      <c r="AK40" s="45"/>
-      <c r="AL40" s="45"/>
-      <c r="AM40" s="45"/>
-      <c r="AN40" s="45"/>
-      <c r="AO40" s="45"/>
-      <c r="AP40" s="45"/>
-      <c r="AQ40" s="45"/>
-      <c r="AR40" s="45"/>
-      <c r="AS40" s="45"/>
-      <c r="AT40" s="45"/>
-      <c r="AU40" s="45"/>
-      <c r="AV40" s="45"/>
-      <c r="AW40" s="45"/>
-      <c r="AX40" s="45"/>
-      <c r="AY40" s="45"/>
-      <c r="AZ40" s="45"/>
-      <c r="BA40" s="45"/>
-      <c r="BB40" s="45"/>
-      <c r="BC40" s="45"/>
-      <c r="BD40" s="45"/>
-      <c r="BE40" s="45"/>
-      <c r="BF40" s="45"/>
-      <c r="BG40" s="45"/>
-      <c r="BH40" s="45"/>
-      <c r="BI40" s="45"/>
-      <c r="BJ40" s="45"/>
-      <c r="BK40" s="45"/>
-      <c r="BL40" s="45"/>
-      <c r="BM40" s="45"/>
+      <c r="J40" s="50"/>
+      <c r="K40" s="50"/>
+      <c r="L40" s="50"/>
+      <c r="M40" s="50"/>
+      <c r="N40" s="50"/>
+      <c r="O40" s="50"/>
+      <c r="P40" s="50"/>
+      <c r="Q40" s="50"/>
+      <c r="R40" s="50"/>
+      <c r="S40" s="50"/>
+      <c r="T40" s="50"/>
+      <c r="U40" s="50"/>
+      <c r="V40" s="50"/>
+      <c r="W40" s="50"/>
+      <c r="X40" s="50"/>
+      <c r="Y40" s="50"/>
+      <c r="Z40" s="50"/>
+      <c r="AA40" s="50"/>
+      <c r="AB40" s="50"/>
+      <c r="AC40" s="50"/>
+      <c r="AD40" s="50"/>
+      <c r="AE40" s="50"/>
+      <c r="AF40" s="50"/>
+      <c r="AG40" s="50"/>
+      <c r="AH40" s="50"/>
+      <c r="AI40" s="50"/>
+      <c r="AJ40" s="50"/>
+      <c r="AK40" s="50"/>
+      <c r="AL40" s="50"/>
+      <c r="AM40" s="50"/>
+      <c r="AN40" s="50"/>
+      <c r="AO40" s="50"/>
+      <c r="AP40" s="50"/>
+      <c r="AQ40" s="50"/>
+      <c r="AR40" s="50"/>
+      <c r="AS40" s="50"/>
+      <c r="AT40" s="50"/>
+      <c r="AU40" s="50"/>
+      <c r="AV40" s="50"/>
+      <c r="AW40" s="50"/>
+      <c r="AX40" s="50"/>
+      <c r="AY40" s="50"/>
+      <c r="AZ40" s="50"/>
+      <c r="BA40" s="50"/>
+      <c r="BB40" s="50"/>
+      <c r="BC40" s="50"/>
+      <c r="BD40" s="50"/>
+      <c r="BE40" s="50"/>
+      <c r="BF40" s="50"/>
+      <c r="BG40" s="50"/>
+      <c r="BH40" s="50"/>
+      <c r="BI40" s="50"/>
+      <c r="BJ40" s="50"/>
+      <c r="BK40" s="50"/>
+      <c r="BL40" s="50"/>
+      <c r="BM40" s="50"/>
     </row>
     <row r="41" spans="1:65" s="46" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="14"/>
-      <c r="B41" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="C41" s="84"/>
-      <c r="D41" s="85"/>
-      <c r="E41" s="86"/>
-      <c r="F41" s="87"/>
-      <c r="G41" s="87"/>
+      <c r="A41" s="13"/>
+      <c r="B41" s="79"/>
+      <c r="C41" s="80"/>
+      <c r="D41" s="81"/>
+      <c r="E41" s="82"/>
+      <c r="F41" s="82"/>
+      <c r="G41" s="82"/>
       <c r="H41" s="17"/>
-      <c r="I41" s="6" t="str">
+      <c r="I41" s="5" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="J41" s="88"/>
-      <c r="K41" s="88"/>
-      <c r="L41" s="88"/>
-      <c r="M41" s="88"/>
-      <c r="N41" s="88"/>
-      <c r="O41" s="88"/>
-      <c r="P41" s="88"/>
-      <c r="Q41" s="88"/>
-      <c r="R41" s="88"/>
-      <c r="S41" s="88"/>
-      <c r="T41" s="88"/>
-      <c r="U41" s="88"/>
-      <c r="V41" s="88"/>
-      <c r="W41" s="88"/>
-      <c r="X41" s="88"/>
-      <c r="Y41" s="88"/>
-      <c r="Z41" s="88"/>
-      <c r="AA41" s="88"/>
-      <c r="AB41" s="88"/>
-      <c r="AC41" s="88"/>
-      <c r="AD41" s="88"/>
-      <c r="AE41" s="88"/>
-      <c r="AF41" s="88"/>
-      <c r="AG41" s="88"/>
-      <c r="AH41" s="88"/>
-      <c r="AI41" s="88"/>
-      <c r="AJ41" s="88"/>
-      <c r="AK41" s="88"/>
-      <c r="AL41" s="88"/>
-      <c r="AM41" s="88"/>
-      <c r="AN41" s="88"/>
-      <c r="AO41" s="88"/>
-      <c r="AP41" s="88"/>
-      <c r="AQ41" s="88"/>
-      <c r="AR41" s="88"/>
-      <c r="AS41" s="88"/>
-      <c r="AT41" s="88"/>
-      <c r="AU41" s="88"/>
-      <c r="AV41" s="88"/>
-      <c r="AW41" s="88"/>
-      <c r="AX41" s="88"/>
-      <c r="AY41" s="88"/>
-      <c r="AZ41" s="88"/>
-      <c r="BA41" s="88"/>
-      <c r="BB41" s="88"/>
-      <c r="BC41" s="88"/>
-      <c r="BD41" s="88"/>
-      <c r="BE41" s="88"/>
-      <c r="BF41" s="88"/>
-      <c r="BG41" s="88"/>
-      <c r="BH41" s="88"/>
-      <c r="BI41" s="88"/>
-      <c r="BJ41" s="88"/>
-      <c r="BK41" s="88"/>
-      <c r="BL41" s="88"/>
-      <c r="BM41" s="88"/>
-    </row>
-    <row r="42" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="H42" s="3"/>
+      <c r="J41" s="45"/>
+      <c r="K41" s="45"/>
+      <c r="L41" s="45"/>
+      <c r="M41" s="45"/>
+      <c r="N41" s="45"/>
+      <c r="O41" s="45"/>
+      <c r="P41" s="45"/>
+      <c r="Q41" s="45"/>
+      <c r="R41" s="45"/>
+      <c r="S41" s="45"/>
+      <c r="T41" s="45"/>
+      <c r="U41" s="45"/>
+      <c r="V41" s="45"/>
+      <c r="W41" s="45"/>
+      <c r="X41" s="45"/>
+      <c r="Y41" s="45"/>
+      <c r="Z41" s="45"/>
+      <c r="AA41" s="45"/>
+      <c r="AB41" s="45"/>
+      <c r="AC41" s="45"/>
+      <c r="AD41" s="45"/>
+      <c r="AE41" s="45"/>
+      <c r="AF41" s="45"/>
+      <c r="AG41" s="45"/>
+      <c r="AH41" s="45"/>
+      <c r="AI41" s="45"/>
+      <c r="AJ41" s="45"/>
+      <c r="AK41" s="45"/>
+      <c r="AL41" s="45"/>
+      <c r="AM41" s="45"/>
+      <c r="AN41" s="45"/>
+      <c r="AO41" s="45"/>
+      <c r="AP41" s="45"/>
+      <c r="AQ41" s="45"/>
+      <c r="AR41" s="45"/>
+      <c r="AS41" s="45"/>
+      <c r="AT41" s="45"/>
+      <c r="AU41" s="45"/>
+      <c r="AV41" s="45"/>
+      <c r="AW41" s="45"/>
+      <c r="AX41" s="45"/>
+      <c r="AY41" s="45"/>
+      <c r="AZ41" s="45"/>
+      <c r="BA41" s="45"/>
+      <c r="BB41" s="45"/>
+      <c r="BC41" s="45"/>
+      <c r="BD41" s="45"/>
+      <c r="BE41" s="45"/>
+      <c r="BF41" s="45"/>
+      <c r="BG41" s="45"/>
+      <c r="BH41" s="45"/>
+      <c r="BI41" s="45"/>
+      <c r="BJ41" s="45"/>
+      <c r="BK41" s="45"/>
+      <c r="BL41" s="45"/>
+      <c r="BM41" s="45"/>
+    </row>
+    <row r="42" spans="1:65" s="46" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="14"/>
+      <c r="B42" s="83" t="s">
+        <v>0</v>
+      </c>
+      <c r="C42" s="84"/>
+      <c r="D42" s="85"/>
+      <c r="E42" s="86"/>
+      <c r="F42" s="87"/>
+      <c r="G42" s="87"/>
+      <c r="H42" s="17"/>
+      <c r="I42" s="6" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="J42" s="88"/>
+      <c r="K42" s="88"/>
+      <c r="L42" s="88"/>
+      <c r="M42" s="88"/>
+      <c r="N42" s="88"/>
+      <c r="O42" s="88"/>
+      <c r="P42" s="88"/>
+      <c r="Q42" s="88"/>
+      <c r="R42" s="88"/>
+      <c r="S42" s="88"/>
+      <c r="T42" s="88"/>
+      <c r="U42" s="88"/>
+      <c r="V42" s="88"/>
+      <c r="W42" s="88"/>
+      <c r="X42" s="88"/>
+      <c r="Y42" s="88"/>
+      <c r="Z42" s="88"/>
+      <c r="AA42" s="88"/>
+      <c r="AB42" s="88"/>
+      <c r="AC42" s="88"/>
+      <c r="AD42" s="88"/>
+      <c r="AE42" s="88"/>
+      <c r="AF42" s="88"/>
+      <c r="AG42" s="88"/>
+      <c r="AH42" s="88"/>
+      <c r="AI42" s="88"/>
+      <c r="AJ42" s="88"/>
+      <c r="AK42" s="88"/>
+      <c r="AL42" s="88"/>
+      <c r="AM42" s="88"/>
+      <c r="AN42" s="88"/>
+      <c r="AO42" s="88"/>
+      <c r="AP42" s="88"/>
+      <c r="AQ42" s="88"/>
+      <c r="AR42" s="88"/>
+      <c r="AS42" s="88"/>
+      <c r="AT42" s="88"/>
+      <c r="AU42" s="88"/>
+      <c r="AV42" s="88"/>
+      <c r="AW42" s="88"/>
+      <c r="AX42" s="88"/>
+      <c r="AY42" s="88"/>
+      <c r="AZ42" s="88"/>
+      <c r="BA42" s="88"/>
+      <c r="BB42" s="88"/>
+      <c r="BC42" s="88"/>
+      <c r="BD42" s="88"/>
+      <c r="BE42" s="88"/>
+      <c r="BF42" s="88"/>
+      <c r="BG42" s="88"/>
+      <c r="BH42" s="88"/>
+      <c r="BI42" s="88"/>
+      <c r="BJ42" s="88"/>
+      <c r="BK42" s="88"/>
+      <c r="BL42" s="88"/>
+      <c r="BM42" s="88"/>
     </row>
     <row r="43" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C43" s="16"/>
-      <c r="F43" s="15"/>
-      <c r="G43" s="15"/>
+      <c r="H43" s="3"/>
     </row>
     <row r="44" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C44" s="4"/>
+      <c r="C44" s="16"/>
+      <c r="F44" s="15"/>
+      <c r="G44" s="15"/>
+    </row>
+    <row r="45" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C45" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="20">
@@ -5407,6 +5494,8 @@
     <mergeCell ref="E5:E6"/>
     <mergeCell ref="D5:D6"/>
     <mergeCell ref="B2:C2"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="R2:AA2"/>
     <mergeCell ref="BG4:BM4"/>
     <mergeCell ref="J4:P4"/>
     <mergeCell ref="Q4:W4"/>
@@ -5415,11 +5504,9 @@
     <mergeCell ref="AL4:AR4"/>
     <mergeCell ref="AS4:AY4"/>
     <mergeCell ref="AZ4:BF4"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="R2:AA2"/>
   </mergeCells>
   <phoneticPr fontId="33" type="noConversion"/>
-  <conditionalFormatting sqref="D7:D41">
+  <conditionalFormatting sqref="D7:D42">
     <cfRule type="dataBar" priority="23">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5433,7 +5520,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J4:BM39">
+  <conditionalFormatting sqref="J4:BM40">
     <cfRule type="expression" dxfId="8" priority="1">
       <formula>AND(TODAY()&gt;=J$5, TODAY()&lt;K$5)</formula>
     </cfRule>
@@ -5454,7 +5541,7 @@
       <formula>AND(task_end&gt;=J$5,task_start&lt;K$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J27:BM33">
+  <conditionalFormatting sqref="J27:BM34">
     <cfRule type="expression" dxfId="3" priority="2">
       <formula>AND(task_start&lt;=J$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=J$5)</formula>
     </cfRule>
@@ -5462,7 +5549,7 @@
       <formula>AND(task_end&gt;=J$5,task_start&lt;K$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J35:BM39">
+  <conditionalFormatting sqref="J36:BM40">
     <cfRule type="expression" dxfId="1" priority="36">
       <formula>AND(task_start&lt;=J$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=J$5)</formula>
     </cfRule>
@@ -5484,8 +5571,8 @@
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Rows 10 through 13 repeat the pattern from row 9. _x000a__x000a_Repeat the instructions from cell A9 for all task rows in this worksheet. _x000a__x000a_Continue entering tasks in cells A10 through A13 or go to cell A14 to learn more." sqref="A10" xr:uid="{872449A7-C3CC-45B6-BA90-B1AAD66BA0E5}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Cell B14 contains the Phase 2 sample title. Enter a new title in cell B14._x000a_To delete the phase and work only from tasks, simply delete this row. To remove the phase, simply delete the row. Add tasks to previous phase by entering a new row above this one._x000a_" sqref="A14" xr:uid="{4F48FC41-E335-47F1-87AA-3333A52AD81C}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Phase 3's sample block starts in cell B20." sqref="A26" xr:uid="{956902D1-D3B5-416D-BB69-9362D193BC0A}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Phase 4's sample block starts in cell B26." sqref="A34" xr:uid="{DE54E5DE-526D-4D71-8D03-E99B4AB2FEE5}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="This row marks the end of the Project Schedule. DO NOT enter anything in this row. _x000a_Insert new rows ABOVE this one to continue building out your Project Schedule." sqref="A41" xr:uid="{79B9237E-4DD3-4E0F-8ED6-E0B695A99D96}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Phase 4's sample block starts in cell B26." sqref="A35" xr:uid="{DE54E5DE-526D-4D71-8D03-E99B4AB2FEE5}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="This row marks the end of the Project Schedule. DO NOT enter anything in this row. _x000a_Insert new rows ABOVE this one to continue building out your Project Schedule." sqref="A42" xr:uid="{79B9237E-4DD3-4E0F-8ED6-E0B695A99D96}"/>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.35" right="0.35" top="0.35" bottom="0.5" header="0.3" footer="0.3"/>
@@ -5542,7 +5629,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>D7:D41</xm:sqref>
+          <xm:sqref>D7:D42</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -5672,15 +5759,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
@@ -5700,7 +5778,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="28" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="60f5a4f2d2b0abadcf532d48ebf9cb71">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7dd78129e6a1811f84807ad11c651531" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -6012,15 +6090,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97245281-08F3-4104-84BD-39F3D8CFB195}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A82239A0-E68C-493F-BEE6-C77FEA397FD6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -6039,7 +6118,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A09426A3-87E9-4865-8A6C-3456B026AE03}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6060,6 +6139,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97245281-08F3-4104-84BD-39F3D8CFB195}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata"/>
 </file>
</xml_diff>